<commit_message>
Implementacion de filtrado de heuristica 1 con zips
</commit_message>
<xml_diff>
--- a/benchmark_Results/benchmark_h1_h2_comparison_simple.xlsx
+++ b/benchmark_Results/benchmark_h1_h2_comparison_simple.xlsx
@@ -932,7 +932,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1184,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
@@ -6875,7 +6875,7 @@
         <v>0</v>
       </c>
       <c r="D307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E307" t="n">
         <v>0</v>
@@ -6959,7 +6959,7 @@
         <v>0</v>
       </c>
       <c r="D311" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E311" t="n">
         <v>0</v>
@@ -9080,7 +9080,7 @@
         <v>1</v>
       </c>
       <c r="D412" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E412" t="n">
         <v>0</v>
@@ -9122,7 +9122,7 @@
         <v>1</v>
       </c>
       <c r="D414" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E414" t="n">
         <v>0</v>
@@ -9143,7 +9143,7 @@
         <v>1</v>
       </c>
       <c r="D415" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E415" t="n">
         <v>1</v>
@@ -9164,7 +9164,7 @@
         <v>1</v>
       </c>
       <c r="D416" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E416" t="n">
         <v>1</v>
@@ -9248,7 +9248,7 @@
         <v>1</v>
       </c>
       <c r="D420" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E420" t="n">
         <v>1</v>
@@ -9269,7 +9269,7 @@
         <v>1</v>
       </c>
       <c r="D421" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E421" t="n">
         <v>1</v>
@@ -9311,7 +9311,7 @@
         <v>1</v>
       </c>
       <c r="D423" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E423" t="n">
         <v>1</v>
@@ -9332,7 +9332,7 @@
         <v>1</v>
       </c>
       <c r="D424" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E424" t="n">
         <v>1</v>
@@ -9353,7 +9353,7 @@
         <v>1</v>
       </c>
       <c r="D425" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E425" t="n">
         <v>1</v>
@@ -9395,7 +9395,7 @@
         <v>1</v>
       </c>
       <c r="D427" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E427" t="n">
         <v>1</v>
@@ -9521,7 +9521,7 @@
         <v>1</v>
       </c>
       <c r="D433" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E433" t="n">
         <v>1</v>
@@ -9920,7 +9920,7 @@
         <v>0</v>
       </c>
       <c r="D452" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E452" t="n">
         <v>0</v>
@@ -10256,7 +10256,7 @@
         <v>0</v>
       </c>
       <c r="D468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E468" t="n">
         <v>0</v>
@@ -10298,7 +10298,7 @@
         <v>0</v>
       </c>
       <c r="D470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E470" t="n">
         <v>0</v>
@@ -10319,7 +10319,7 @@
         <v>1</v>
       </c>
       <c r="D471" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E471" t="n">
         <v>0</v>
@@ -11348,7 +11348,7 @@
         <v>1</v>
       </c>
       <c r="D520" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E520" t="n">
         <v>0</v>
@@ -11495,7 +11495,7 @@
         <v>1</v>
       </c>
       <c r="D527" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E527" t="n">
         <v>0</v>
@@ -11579,7 +11579,7 @@
         <v>1</v>
       </c>
       <c r="D531" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E531" t="n">
         <v>0</v>
@@ -11684,7 +11684,7 @@
         <v>1</v>
       </c>
       <c r="D536" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E536" t="n">
         <v>0</v>
@@ -11852,7 +11852,7 @@
         <v>0</v>
       </c>
       <c r="D544" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E544" t="n">
         <v>0</v>
@@ -11873,7 +11873,7 @@
         <v>1</v>
       </c>
       <c r="D545" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E545" t="n">
         <v>1</v>

</xml_diff>